<commit_message>
Sunrise Rye Brook: vendor RFQ rev 1, all electric heat 208V/3ph
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Avx13TP2m6NHdmoZVrM4Ph
</commit_message>
<xml_diff>
--- a/Reference/Projects/Sunrise Rye Brook - 900 King St/VE Vendor RFQ/VE Vendor RFQ - Sunrise Rye Brook.xlsx
+++ b/Reference/Projects/Sunrise Rye Brook - 900 King St/VE Vendor RFQ/VE Vendor RFQ - Sunrise Rye Brook.xlsx
@@ -474,14 +474,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sunrise Rye Brook - VE request for pricing Rev 0 10/6/2026 - Northern Wolves AC</t>
+          <t>Sunrise Rye Brook - VE request for pricing Rev 1 10/6/2026 - Northern Wolves AC</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Fill in unit price and lead time. Electric heat: 277 V/1 ph up to 5 kW, 480 V/3 ph above (to be confirmed).</t>
+          <t>Fill in unit price and lead time. Electric heat: all 208 V / 3 ph, kW rated at 208 V (note any item only available 208 V / 1 ph).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sunrise Rye Brook: vendor RFQ - VAV coils up to 5 kW at 208V/1ph, voltage per box
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Avx13TP2m6NHdmoZVrM4Ph
</commit_message>
<xml_diff>
--- a/Reference/Projects/Sunrise Rye Brook - 900 King St/VE Vendor RFQ/VE Vendor RFQ - Sunrise Rye Brook.xlsx
+++ b/Reference/Projects/Sunrise Rye Brook - 900 King St/VE Vendor RFQ/VE Vendor RFQ - Sunrise Rye Brook.xlsx
@@ -481,7 +481,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Fill in unit price and lead time. Electric heat: all 208 V / 3 ph, kW rated at 208 V (note any item only available 208 V / 1 ph).</t>
+          <t>Fill in unit price and lead time. Electric heat at 208 V (kW rated at 208 V): VAV coils per Volts column, heaters 208 V / 3 ph.</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Notes / volts</t>
         </is>
       </c>
     </row>
@@ -599,6 +599,11 @@
         <f>IF(J6="","",H6*J6)</f>
         <v/>
       </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -640,6 +645,11 @@
         <f>IF(J7="","",H7*J7)</f>
         <v/>
       </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -681,6 +691,11 @@
         <f>IF(J8="","",H8*J8)</f>
         <v/>
       </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -722,6 +737,11 @@
         <f>IF(J9="","",H9*J9)</f>
         <v/>
       </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -763,6 +783,11 @@
         <f>IF(J10="","",H10*J10)</f>
         <v/>
       </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -804,6 +829,11 @@
         <f>IF(J11="","",H11*J11)</f>
         <v/>
       </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -845,6 +875,11 @@
         <f>IF(J12="","",H12*J12)</f>
         <v/>
       </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -886,6 +921,11 @@
         <f>IF(J13="","",H13*J13)</f>
         <v/>
       </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -927,6 +967,11 @@
         <f>IF(J14="","",H14*J14)</f>
         <v/>
       </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -968,6 +1013,11 @@
         <f>IF(J15="","",H15*J15)</f>
         <v/>
       </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1009,6 +1059,11 @@
         <f>IF(J16="","",H16*J16)</f>
         <v/>
       </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1056,6 +1111,11 @@
         <f>IF(J17="","",H17*J17)</f>
         <v/>
       </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1097,6 +1157,11 @@
         <f>IF(J18="","",H18*J18)</f>
         <v/>
       </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1138,6 +1203,11 @@
         <f>IF(J19="","",H19*J19)</f>
         <v/>
       </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1179,6 +1249,11 @@
         <f>IF(J20="","",H20*J20)</f>
         <v/>
       </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1220,6 +1295,11 @@
         <f>IF(J21="","",H21*J21)</f>
         <v/>
       </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1261,6 +1341,11 @@
         <f>IF(J22="","",H22*J22)</f>
         <v/>
       </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1302,6 +1387,11 @@
         <f>IF(J23="","",H23*J23)</f>
         <v/>
       </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -1343,6 +1433,11 @@
         <f>IF(J24="","",H24*J24)</f>
         <v/>
       </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1384,6 +1479,11 @@
         <f>IF(J25="","",H25*J25)</f>
         <v/>
       </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -1425,6 +1525,11 @@
         <f>IF(J26="","",H26*J26)</f>
         <v/>
       </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1466,6 +1571,11 @@
         <f>IF(J27="","",H27*J27)</f>
         <v/>
       </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -1507,6 +1617,11 @@
         <f>IF(J28="","",H28*J28)</f>
         <v/>
       </c>
+      <c r="M28" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -1548,6 +1663,11 @@
         <f>IF(J29="","",H29*J29)</f>
         <v/>
       </c>
+      <c r="M29" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -1589,6 +1709,11 @@
         <f>IF(J30="","",H30*J30)</f>
         <v/>
       </c>
+      <c r="M30" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -1629,6 +1754,11 @@
       <c r="K31" s="5">
         <f>IF(J31="","",H31*J31)</f>
         <v/>
+      </c>
+      <c r="M31" s="5" t="inlineStr">
+        <is>
+          <t>208/1</t>
+        </is>
       </c>
     </row>
     <row r="32"/>
@@ -1702,7 +1832,7 @@
       </c>
       <c r="M34" s="3" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Notes / volts</t>
         </is>
       </c>
     </row>
@@ -1933,7 +2063,7 @@
       </c>
       <c r="M41" s="3" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Notes / volts</t>
         </is>
       </c>
     </row>
@@ -2710,7 +2840,7 @@
       </c>
       <c r="M62" s="3" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Notes / volts</t>
         </is>
       </c>
     </row>
@@ -2752,6 +2882,11 @@
         <f>IF(J63="","",H63*J63)</f>
         <v/>
       </c>
+      <c r="M63" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -2791,6 +2926,11 @@
         <f>IF(J64="","",H64*J64)</f>
         <v/>
       </c>
+      <c r="M64" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
@@ -2830,6 +2970,11 @@
         <f>IF(J65="","",H65*J65)</f>
         <v/>
       </c>
+      <c r="M65" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
@@ -2869,6 +3014,11 @@
         <f>IF(J66="","",H66*J66)</f>
         <v/>
       </c>
+      <c r="M66" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
@@ -2908,6 +3058,11 @@
         <f>IF(J67="","",H67*J67)</f>
         <v/>
       </c>
+      <c r="M67" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
@@ -2947,6 +3102,11 @@
         <f>IF(J68="","",H68*J68)</f>
         <v/>
       </c>
+      <c r="M68" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
@@ -2986,6 +3146,11 @@
         <f>IF(J69="","",H69*J69)</f>
         <v/>
       </c>
+      <c r="M69" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
@@ -3025,6 +3190,11 @@
         <f>IF(J70="","",H70*J70)</f>
         <v/>
       </c>
+      <c r="M70" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
@@ -3064,6 +3234,11 @@
         <f>IF(J71="","",H71*J71)</f>
         <v/>
       </c>
+      <c r="M71" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
@@ -3103,6 +3278,11 @@
         <f>IF(J72="","",H72*J72)</f>
         <v/>
       </c>
+      <c r="M72" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="73"/>
     <row r="74">
@@ -3175,7 +3355,7 @@
       </c>
       <c r="M75" s="3" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Notes / volts</t>
         </is>
       </c>
     </row>
@@ -3213,6 +3393,11 @@
         <f>IF(J76="","",H76*J76)</f>
         <v/>
       </c>
+      <c r="M76" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
@@ -3248,6 +3433,11 @@
         <f>IF(J77="","",H77*J77)</f>
         <v/>
       </c>
+      <c r="M77" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
@@ -3283,6 +3473,11 @@
         <f>IF(J78="","",H78*J78)</f>
         <v/>
       </c>
+      <c r="M78" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
@@ -3318,6 +3513,11 @@
         <f>IF(J79="","",H79*J79)</f>
         <v/>
       </c>
+      <c r="M79" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
@@ -3353,6 +3553,11 @@
         <f>IF(J80="","",H80*J80)</f>
         <v/>
       </c>
+      <c r="M80" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
@@ -3388,6 +3593,11 @@
         <f>IF(J81="","",H81*J81)</f>
         <v/>
       </c>
+      <c r="M81" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
@@ -3423,6 +3633,11 @@
         <f>IF(J82="","",H82*J82)</f>
         <v/>
       </c>
+      <c r="M82" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
@@ -3458,6 +3673,11 @@
         <f>IF(J83="","",H83*J83)</f>
         <v/>
       </c>
+      <c r="M83" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
@@ -3493,6 +3713,11 @@
         <f>IF(J84="","",H84*J84)</f>
         <v/>
       </c>
+      <c r="M84" s="5" t="inlineStr">
+        <is>
+          <t>208/3</t>
+        </is>
+      </c>
     </row>
     <row r="85"/>
     <row r="86">
@@ -3565,7 +3790,7 @@
       </c>
       <c r="M87" s="3" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Notes / volts</t>
         </is>
       </c>
     </row>
@@ -3988,7 +4213,7 @@
       </c>
       <c r="M102" s="3" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Notes / volts</t>
         </is>
       </c>
     </row>

</xml_diff>